<commit_message>
Add validated Phase 1 workflow and adjusted HAZUS repair cost ratios
</commit_message>
<xml_diff>
--- a/data/reference/hazus/repair_cost_ratios/HAZUS_Drift_Sensitive_Nonstructural_Repair_Costs.xlsx
+++ b/data/reference/hazus/repair_cost_ratios/HAZUS_Drift_Sensitive_Nonstructural_Repair_Costs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\randlee\Box\Randle_Emmanuel\NSI_Oregon\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\seismic-correlation-insurance-loss\data\reference\hazus\repair_cost_ratios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C43654D-484D-42DD-BE51-557E6A844B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355C29C5-4E08-4D40-BBCA-9844D7C1EEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -976,7 +976,7 @@
         <v>17.8</v>
       </c>
       <c r="F19">
-        <v>35.5</v>
+        <v>34.4</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
@@ -996,7 +996,7 @@
         <v>17.8</v>
       </c>
       <c r="F20">
-        <v>35.4</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>